<commit_message>
Refresh nilai evaluasi BPH dari live sheets: update ranking Best Department
</commit_message>
<xml_diff>
--- a/PA_September_2026_Rekapitulasi_Lengkap.xlsx
+++ b/PA_September_2026_Rekapitulasi_Lengkap.xlsx
@@ -759,22 +759,22 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Departemen Dalam Negeri</t>
+          <t>Departemen Pengembangan Sumber Daya Mahasiswa</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>DAGRI</t>
+          <t>PSDM</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>8.6</v>
+        <v>8.56</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>8.550000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>8.630000000000001</v>
+        <v>8.16</v>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
@@ -783,12 +783,12 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>15 Fungsionaris</t>
+          <t>13 Fungsionaris</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>Ilman Afif Al Arif: 8.3, Muhammad Mirza Zaidan 'Ilma: 8.8</t>
+          <t>Ilman Afif Al Arif: 9.8, Muhammad Mirza Zaidan 'Ilma: 9.2, Bramantio Ramayudha: 9.5</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
@@ -805,22 +805,22 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Departemen Pengembangan Sumber Daya Mahasiswa</t>
+          <t>Departemen Dalam Negeri</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>PSDM</t>
+          <t>DAGRI</t>
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>8.49</v>
+        <v>8.48</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>9.27</v>
+        <v>8.15</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>8.16</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
@@ -829,12 +829,12 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>13 Fungsionaris</t>
+          <t>15 Fungsionaris</t>
         </is>
       </c>
       <c r="I8" s="18" t="inlineStr">
         <is>
-          <t>Ilman Afif Al Arif: 9.8, Muhammad Mirza Zaidan 'Ilma: 8.5, Bramantio Ramayudha: 9.5</t>
+          <t>Ilman Afif Al Arif: 8.3, Muhammad Mirza Zaidan 'Ilma: 8.0</t>
         </is>
       </c>
       <c r="J8" s="14" t="inlineStr">

</xml_diff>